<commit_message>
fix(excel): merge two separated tables#2626, follow-up fix test issues
Signed-off-by: Michele-Zhu <michele.zhu@polimi.it>
</commit_message>
<xml_diff>
--- a/tests/data/xlsx/xlsx_07_table_with_missing_header_middle.xlsx
+++ b/tests/data/xlsx/xlsx_07_table_with_missing_header_middle.xlsx
@@ -5,11 +5,10 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
   <si>
     <t xml:space="preserve">Product/Integration</t>
   </si>
@@ -601,115 +600,4 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData>
-    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
-  </headerFooter>
-</worksheet>
 </file>
</xml_diff>